<commit_message>
fix(import): handle excel serial dates and generate separate entity files
</commit_message>
<xml_diff>
--- a/test-data/payments.xlsx
+++ b/test-data/payments.xlsx
@@ -397,35 +397,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Fecha</v>
       </c>
       <c r="B1" t="str">
-        <v>Tipo</v>
+        <v>Entidad</v>
       </c>
       <c r="C1" t="str">
         <v>Monto</v>
       </c>
       <c r="D1" t="str">
-        <v>ID Referencia</v>
+        <v>Tipo</v>
       </c>
       <c r="E1" t="str">
-        <v>Doc Vinculado</v>
+        <v>Método</v>
       </c>
       <c r="F1" t="str">
-        <v>Medio de Pago</v>
-      </c>
-      <c r="G1" t="str">
         <v>Banco</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Ref Instrumento</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Disponibilidad</v>
       </c>
     </row>
     <row r="2">
@@ -433,120 +424,84 @@
         <v>10/01/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>OP</v>
+        <v>Cliente Alpha S.A.</v>
       </c>
       <c r="C2">
-        <v>100000</v>
+        <v>350000</v>
       </c>
       <c r="D2" t="str">
-        <v>OP-102</v>
+        <v>Cobro</v>
       </c>
       <c r="E2" t="str">
-        <v>Factura Inmobiliaria (Ene)</v>
+        <v>Transferencia</v>
       </c>
       <c r="F2" t="str">
-        <v>transferencia</v>
-      </c>
-      <c r="G2" t="str">
         <v>Galicia</v>
-      </c>
-      <c r="H2" t="str">
-        <v>TRF-9981</v>
-      </c>
-      <c r="I2" t="str">
-        <v>10/01/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>15/01/2026</v>
+        <v>12/01/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>Recibo</v>
+        <v>Inmobiliaria Local</v>
       </c>
       <c r="C3">
-        <v>350000</v>
+        <v>100000</v>
       </c>
       <c r="D3" t="str">
-        <v>REC-501</v>
+        <v>Pago</v>
       </c>
       <c r="E3" t="str">
-        <v>Fact-A-201 (Alpha)</v>
+        <v>Efectivo</v>
       </c>
       <c r="F3" t="str">
-        <v>cheque_terceros</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Santander</v>
-      </c>
-      <c r="H3" t="str">
-        <v>CH-4401</v>
-      </c>
-      <c r="I3" t="str">
-        <v>30/01/2026</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>05/02/2026</v>
+        <v>15/01/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>OP</v>
+        <v>Cliente Beta Corp</v>
       </c>
       <c r="C4">
-        <v>650000</v>
+        <v>450000</v>
       </c>
       <c r="D4" t="str">
-        <v>OP-201</v>
+        <v>Cobro</v>
       </c>
       <c r="E4" t="str">
-        <v>Nómina General</v>
+        <v>Transferencia</v>
       </c>
       <c r="F4" t="str">
-        <v>transferencia</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Galicia</v>
-      </c>
-      <c r="H4" t="str">
-        <v>TRF-2210</v>
-      </c>
-      <c r="I4" t="str">
-        <v>05/02/2026</v>
+        <v>Santander</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>25/02/2026</v>
+        <v>10/02/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>Recibo</v>
+        <v>Cliente Alpha S.A.</v>
       </c>
       <c r="C5">
-        <v>450000</v>
+        <v>350000</v>
       </c>
       <c r="D5" t="str">
-        <v>REC-602</v>
+        <v>Cobro</v>
       </c>
       <c r="E5" t="str">
-        <v>Fact-A-302 (Beta)</v>
+        <v>Transferencia</v>
       </c>
       <c r="F5" t="str">
-        <v>transferencia</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Macro</v>
-      </c>
-      <c r="H5" t="str">
-        <v>TRF-1102</v>
-      </c>
-      <c r="I5" t="str">
-        <v>25/02/2026</v>
+        <v>Galicia</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>